<commit_message>
Refactor bug severity and priority levels based on business impact
</commit_message>
<xml_diff>
--- a/Bug-raports/Bug-raport_Erbology_v.1.0.xlsx
+++ b/Bug-raports/Bug-raport_Erbology_v.1.0.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="FS" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Minor</t>
   </si>
   <si>
-    <t>Low</t>
+    <t>Medium</t>
   </si>
   <si>
     <t xml:space="preserve">When switching the website region to an English-speaking Eurozone country (e.g., Germany), duplicate information blocks appear at the top of the page.</t>
@@ -149,6 +149,9 @@
     <t>Cursor</t>
   </si>
   <si>
+    <t>Low</t>
+  </si>
+  <si>
     <t xml:space="preserve">Missing "cursor: pointer" style on the final "Sign up" registration button.
 </t>
   </si>
@@ -260,6 +263,9 @@
   </si>
   <si>
     <t>Performance</t>
+  </si>
+  <si>
+    <t>Major</t>
   </si>
   <si>
     <t xml:space="preserve">Critical client-side performance degradation and high thread blocking on mobile devices under baseline network conditions (10 Mbps).</t>
@@ -323,7 +329,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="5">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -335,43 +341,6 @@
       <left style="thin">
         <color theme="1"/>
       </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color theme="1"/>
       </right>
@@ -424,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -459,15 +428,6 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1195,7 +1155,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{00CF0084-002B-48D4-BFDA-00A8004300B8}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{007D00D8-0095-4ED6-8082-00A600920064}">
             <xm:f>"Trivial"</xm:f>
             <x14:dxf>
               <font>
@@ -1212,7 +1172,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{0055003B-0022-427E-A577-00020021009B}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{000A0061-0038-4768-A21C-00AF006D006E}">
             <xm:f>"Minor"</xm:f>
             <x14:dxf>
               <font>
@@ -1229,7 +1189,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00C50046-008E-4D43-8C13-009200680086}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00B20077-00B3-46E9-938F-009C009700D3}">
             <xm:f>"Major"</xm:f>
             <x14:dxf>
               <fill>
@@ -1243,7 +1203,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00D0003E-0068-4B50-A873-004300F60006}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{005C00F8-003C-4D71-B3A4-00A9007E009C}">
             <xm:f>"Critical"</xm:f>
             <x14:dxf>
               <font>
@@ -1260,7 +1220,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{005A0002-0039-43F5-9850-000000FB0089}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{008400E7-00FC-461E-9D80-00F500410091}">
             <xm:f>"Blocker"</xm:f>
             <x14:dxf>
               <font>
@@ -1277,7 +1237,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00FB0036-00A1-4E2A-8EDA-003B007E00E5}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00B800E8-0092-4D8F-9116-0005003400C3}">
             <xm:f>"Low"</xm:f>
             <x14:dxf>
               <font>
@@ -1294,7 +1254,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{007F00BF-00D3-4B08-9133-006700D600CF}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{001B00C5-0090-4869-ABAE-003F00600003}">
             <xm:f>"Medium"</xm:f>
             <x14:dxf>
               <font>
@@ -1311,7 +1271,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00660049-0017-404B-82F1-007E00320065}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00E600EB-00FC-49D6-B068-007000000068}">
             <xm:f>"High"</xm:f>
             <x14:dxf>
               <font>
@@ -1328,7 +1288,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{006400C1-0047-42D7-829B-007C001200A5}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{00E200EE-00D0-4A01-A0B4-0047000500CD}">
             <xm:f>"Highest"</xm:f>
             <x14:dxf>
               <font>
@@ -1345,7 +1305,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{00E200DB-0052-4130-9634-00E200CC00F3}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{00EF0001-007B-4C9B-A4D7-00D800920050}">
             <xm:f>"Trivial"</xm:f>
             <x14:dxf>
               <font>
@@ -1362,7 +1322,7 @@
           <xm:sqref>C5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{007B008D-00BC-4E00-A7AD-003400080098}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{0081007E-005E-4759-8469-001A008000D5}">
             <xm:f>"Minor"</xm:f>
             <x14:dxf>
               <font>
@@ -1379,7 +1339,7 @@
           <xm:sqref>C5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00800092-001C-4A95-9169-007B0043003D}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{001D0064-0050-4874-AEDA-006900DC0081}">
             <xm:f>"Major"</xm:f>
             <x14:dxf>
               <fill>
@@ -1393,7 +1353,7 @@
           <xm:sqref>C5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{007400E9-009C-4160-BAC5-00C300500074}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00E000D4-001A-4D28-93E7-00040064003F}">
             <xm:f>"Critical"</xm:f>
             <x14:dxf>
               <font>
@@ -1410,7 +1370,7 @@
           <xm:sqref>C5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00910053-007D-4078-848F-009E00D2002F}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00F90094-00FC-4835-8C2A-0090000E003E}">
             <xm:f>"Blocker"</xm:f>
             <x14:dxf>
               <font>
@@ -1427,7 +1387,7 @@
           <xm:sqref>C5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{004100D8-0091-4415-8586-00A000C40047}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{002A008C-0026-4861-9187-009300810071}">
             <xm:f>"Low"</xm:f>
             <x14:dxf>
               <font>
@@ -1444,7 +1404,7 @@
           <xm:sqref>D5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{00A60042-00BF-4115-96E6-00E100F200F7}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{004B004C-003F-4EF4-87BE-00FA009A000E}">
             <xm:f>"Medium"</xm:f>
             <x14:dxf>
               <font>
@@ -1461,7 +1421,7 @@
           <xm:sqref>D5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{001300A1-0082-4F7A-B0D3-007E007D005E}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00C60083-00E2-463A-94E2-009400E80010}">
             <xm:f>"High"</xm:f>
             <x14:dxf>
               <font>
@@ -1478,7 +1438,7 @@
           <xm:sqref>D5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{009000C5-006A-44EA-96EF-0018005A0000}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{001C0089-001B-4805-89D5-0095003100B5}">
             <xm:f>"Highest"</xm:f>
             <x14:dxf>
               <font>
@@ -1498,25 +1458,25 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4" disablePrompts="0">
-        <x14:dataValidation xr:uid="{005A00C7-0099-4F2E-94CA-005300D30046}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{005F00D6-00EF-4428-9AD0-001400EB0000}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Blocker,Critical,Major,Minor,Trivial"</xm:f>
           </x14:formula1>
           <xm:sqref>C2</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00610081-0047-4EB3-8A6C-0058000500F9}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00B60089-00D1-46FD-A7E2-008D00C30038}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Highest,High,Medium,Low"</xm:f>
           </x14:formula1>
           <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00C80011-003F-410C-88CF-0054006000CB}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00DC00E2-002E-4FE0-956B-006000190067}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Blocker,Critical,Major,Minor,Trivial"</xm:f>
           </x14:formula1>
           <xm:sqref>C5</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0068005A-0060-4B6E-BE60-00F7002A00CE}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00A100C8-00E2-47B2-B4A0-004F008100DC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Highest,High,Medium,Low"</xm:f>
           </x14:formula1>
@@ -1582,19 +1542,19 @@
         <v>11</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -1605,7 +1565,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
       <c r="F3" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -1618,7 +1578,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -1631,7 +1591,7 @@
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -1644,7 +1604,7 @@
       <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
@@ -1657,7 +1617,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -1665,28 +1625,28 @@
     </row>
     <row r="8" ht="57">
       <c r="A8" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I8" s="4"/>
     </row>
@@ -1697,7 +1657,7 @@
       <c r="D9" s="2"/>
       <c r="E9" s="3"/>
       <c r="F9" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -1710,34 +1670,34 @@
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
       <c r="F10" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="14"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="8"/>
     </row>
     <row r="12">
-      <c r="A12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
+      <c r="A12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
     </row>
     <row r="13">
-      <c r="A13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
+      <c r="A13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -1767,7 +1727,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{004D0083-001D-4532-B381-00F600FD00FB}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{00670044-00C1-4757-BC0A-0004004400AA}">
             <xm:f>"Trivial"</xm:f>
             <x14:dxf>
               <font>
@@ -1784,7 +1744,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{00370076-00FE-4257-9707-008A004400AD}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{00A60004-000F-4E38-9009-008900DE0027}">
             <xm:f>"Minor"</xm:f>
             <x14:dxf>
               <font>
@@ -1801,7 +1761,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{001B0062-001C-4DFE-9AC0-00EE00C20023}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{006900D9-0008-48C2-9B4B-00CE007E006D}">
             <xm:f>"Major"</xm:f>
             <x14:dxf>
               <fill>
@@ -1815,7 +1775,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00A0003A-00A9-44EC-9FE7-00E4000C0002}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00D00039-0059-46E5-B754-0027008800DC}">
             <xm:f>"Critical"</xm:f>
             <x14:dxf>
               <font>
@@ -1832,7 +1792,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00A20034-0065-400B-B3AF-0031000900D0}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{008C00BE-00A4-4295-A501-00CB00160096}">
             <xm:f>"Blocker"</xm:f>
             <x14:dxf>
               <font>
@@ -1849,7 +1809,7 @@
           <xm:sqref>C2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00B2004A-002A-4EE9-9BBE-001C0079007A}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{006500A5-0000-464C-94FD-005600730002}">
             <xm:f>"Low"</xm:f>
             <x14:dxf>
               <font>
@@ -1866,7 +1826,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{009400BC-0061-4238-B2AE-00F3006B00CE}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{00B70050-0077-4387-8048-0047009F004A}">
             <xm:f>"Medium"</xm:f>
             <x14:dxf>
               <font>
@@ -1883,7 +1843,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00C0008C-008B-464C-948D-008700C50002}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00F000C5-0087-4945-90BA-008300CE00DD}">
             <xm:f>"High"</xm:f>
             <x14:dxf>
               <font>
@@ -1900,7 +1860,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{00E20000-00B9-4DA0-9B5F-00AB00C1002B}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{0014002C-00A1-4A8B-997A-00D100E800ED}">
             <xm:f>"Highest"</xm:f>
             <x14:dxf>
               <font>
@@ -1917,7 +1877,7 @@
           <xm:sqref>D2</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{005A0024-0014-4B51-AB97-00B9006A00C7}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{003A0055-00AD-44E2-9F86-005C000A00F2}">
             <xm:f>"Trivial"</xm:f>
             <x14:dxf>
               <font>
@@ -1934,7 +1894,7 @@
           <xm:sqref>C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{00BC0046-0056-4DA1-90A1-000C00230034}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{000C002F-0084-46D7-B22D-003400040025}">
             <xm:f>"Minor"</xm:f>
             <x14:dxf>
               <font>
@@ -1951,7 +1911,7 @@
           <xm:sqref>C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00510079-004F-4876-A95C-008700200037}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{004B0052-0074-467B-9399-00CC00DA0006}">
             <xm:f>"Major"</xm:f>
             <x14:dxf>
               <fill>
@@ -1965,7 +1925,7 @@
           <xm:sqref>C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00940012-0061-4FD9-A498-000D00EB0076}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00480076-00BF-47E1-B13E-007D004300D6}">
             <xm:f>"Critical"</xm:f>
             <x14:dxf>
               <font>
@@ -1982,7 +1942,7 @@
           <xm:sqref>C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00B6002D-0004-4277-8D9C-000700E000FE}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{006C00FA-001C-43A2-AC6A-0002002C001E}">
             <xm:f>"Blocker"</xm:f>
             <x14:dxf>
               <font>
@@ -1999,7 +1959,7 @@
           <xm:sqref>C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{001A0029-0043-4423-A8A2-00E100B200BE}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00B1005E-0035-4D5C-B2C1-00FB00360026}">
             <xm:f>"Low"</xm:f>
             <x14:dxf>
               <font>
@@ -2016,7 +1976,7 @@
           <xm:sqref>D8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{00DA0028-003C-4852-9F59-008D00E40009}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{002700C9-0028-4A2E-A6B7-006B0034007F}">
             <xm:f>"Medium"</xm:f>
             <x14:dxf>
               <font>
@@ -2033,7 +1993,7 @@
           <xm:sqref>D8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00400090-00A4-4C9E-BD62-00FE00500018}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00700085-0007-473E-9814-003900AE007A}">
             <xm:f>"High"</xm:f>
             <x14:dxf>
               <font>
@@ -2050,7 +2010,7 @@
           <xm:sqref>D8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{004E008D-0041-4344-BCD4-00AE00A30086}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{0044007D-0057-4033-8C76-00B2006000AF}">
             <xm:f>"Highest"</xm:f>
             <x14:dxf>
               <font>
@@ -2070,25 +2030,25 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4" disablePrompts="0">
-        <x14:dataValidation xr:uid="{0037008C-006F-4DA5-A2B8-001900DF00D2}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00EE00C6-0094-45BB-97CC-000600BC0077}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Blocker,Critical,Major,Minor,Trivial"</xm:f>
           </x14:formula1>
           <xm:sqref>C2</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00E300C1-009C-46C9-AB8E-004000D800E1}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00CD0013-00AC-4407-84DE-00C600640071}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Highest,High,Medium,Low"</xm:f>
           </x14:formula1>
           <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{006F00A3-00CC-4DD7-87C6-002700B80079}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00D4003F-007F-494A-8DC5-006D00B10001}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Blocker,Critical,Major,Minor,Trivial"</xm:f>
           </x14:formula1>
           <xm:sqref>C8</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00AA006B-0015-409E-A848-0057007B00C7}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{000A00C7-0066-4C3E-A46C-00D4002F00CC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Highest,High,Medium,Low"</xm:f>
           </x14:formula1>
@@ -2143,28 +2103,28 @@
     </row>
     <row r="2" ht="71.25">
       <c r="A2" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -2175,7 +2135,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
       <c r="F3" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -2188,7 +2148,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -2201,7 +2161,7 @@
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -2209,28 +2169,28 @@
     </row>
     <row r="6" ht="71.25">
       <c r="A6" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -2241,7 +2201,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -2254,7 +2214,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="3"/>
       <c r="F8" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
@@ -2267,7 +2227,7 @@
       <c r="D9" s="2"/>
       <c r="E9" s="3"/>
       <c r="F9" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -2280,7 +2240,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
       <c r="F10" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -2293,7 +2253,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
       <c r="F11" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -2301,31 +2261,31 @@
     </row>
     <row r="12" ht="85.5">
       <c r="A12" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" ht="85.5">
@@ -2335,7 +2295,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
       <c r="F13" s="10" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -2348,7 +2308,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="3"/>
       <c r="F14" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
@@ -2361,7 +2321,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="3"/>
       <c r="F15" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
@@ -2374,24 +2334,24 @@
       <c r="D16" s="2"/>
       <c r="E16" s="3"/>
       <c r="F16" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="14"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -2429,7 +2389,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{00990098-0023-4610-9AEC-005D007300DA}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{000A004D-00A9-429F-8B17-00BB001E003D}">
             <xm:f>"Trivial"</xm:f>
             <x14:dxf>
               <font>
@@ -2446,7 +2406,7 @@
           <xm:sqref>C2 C6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{00F4006E-00B5-48C1-B702-004900C60025}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{00850016-0007-47AD-BCD8-004700F20004}">
             <xm:f>"Minor"</xm:f>
             <x14:dxf>
               <font>
@@ -2463,7 +2423,7 @@
           <xm:sqref>C2 C6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00A70072-001F-416C-99CC-002F00EB0001}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00BB008D-0031-42AE-A61A-007F00D40092}">
             <xm:f>"Major"</xm:f>
             <x14:dxf>
               <fill>
@@ -2477,7 +2437,7 @@
           <xm:sqref>C2 C6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{005300EF-00C6-416F-B2FE-00AA00300029}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{000600BF-004F-4D6A-AD19-00CE0020009E}">
             <xm:f>"Critical"</xm:f>
             <x14:dxf>
               <font>
@@ -2494,7 +2454,7 @@
           <xm:sqref>C2 C6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00CA0075-00A7-4D4A-A144-00540037003C}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{004F00DC-007B-4AAE-8A66-008400E500A3}">
             <xm:f>"Blocker"</xm:f>
             <x14:dxf>
               <font>
@@ -2511,7 +2471,7 @@
           <xm:sqref>C2 C6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00960055-00D1-4723-9EBE-004F0074003F}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{009600BC-0041-4CCA-B16A-00550067005F}">
             <xm:f>"Low"</xm:f>
             <x14:dxf>
               <font>
@@ -2528,7 +2488,7 @@
           <xm:sqref>D2 D6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{00730026-00E6-4945-BD79-00C000B00018}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{006F0058-0025-4C12-88D8-00D800A00055}">
             <xm:f>"Medium"</xm:f>
             <x14:dxf>
               <font>
@@ -2545,7 +2505,7 @@
           <xm:sqref>D2 D6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00D00043-009D-409D-B401-004E00890014}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{007F004C-001C-4D60-B341-000900BB004C}">
             <xm:f>"High"</xm:f>
             <x14:dxf>
               <font>
@@ -2562,7 +2522,7 @@
           <xm:sqref>D2 D6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{0052004A-0043-473C-B9CA-00A700F00062}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{0003005C-0012-4890-A787-00C8009800CE}">
             <xm:f>"Highest"</xm:f>
             <x14:dxf>
               <font>
@@ -2579,7 +2539,7 @@
           <xm:sqref>D2 D6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{0050009E-0036-4ED8-B3C7-00FB00AA0095}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{004A00EC-0063-4F03-995B-0057004B00AB}">
             <xm:f>"Trivial"</xm:f>
             <x14:dxf>
               <font>
@@ -2596,7 +2556,7 @@
           <xm:sqref>C12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{005800E6-0068-4B4B-B0D9-007F00D00026}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{00360086-0062-421D-B1CB-00E0009C0073}">
             <xm:f>"Minor"</xm:f>
             <x14:dxf>
               <font>
@@ -2613,7 +2573,7 @@
           <xm:sqref>C12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00A9008C-00E2-4D11-B655-00EC005000F0}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{00BF0058-00D5-49C8-97B0-00ED008800FF}">
             <xm:f>"Major"</xm:f>
             <x14:dxf>
               <fill>
@@ -2627,7 +2587,7 @@
           <xm:sqref>C12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{00B7003F-003F-4BCE-9C87-00FD006900B2}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{006F00B3-0076-4AEE-883D-00EE00BF00E9}">
             <xm:f>"Critical"</xm:f>
             <x14:dxf>
               <font>
@@ -2644,7 +2604,7 @@
           <xm:sqref>C12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00AB0072-002C-40C7-BB2A-00F500320091}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{00E7008E-0073-4E02-BF77-00B70024000F}">
             <xm:f>"Blocker"</xm:f>
             <x14:dxf>
               <font>
@@ -2661,7 +2621,7 @@
           <xm:sqref>C12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00E000DB-00EF-4164-A5F2-001600140093}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{00590000-00F0-4578-B0B7-00FF00510014}">
             <xm:f>"Low"</xm:f>
             <x14:dxf>
               <font>
@@ -2678,7 +2638,7 @@
           <xm:sqref>D12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{006700F5-00DD-49B4-B907-002B004B0025}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{000C00CA-0080-4449-8F29-00E3001000DF}">
             <xm:f>"Medium"</xm:f>
             <x14:dxf>
               <font>
@@ -2695,7 +2655,7 @@
           <xm:sqref>D12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{0083007E-00E2-46E9-B57E-00FF00690096}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{00DB00CB-00B0-4470-A652-006000E2001A}">
             <xm:f>"High"</xm:f>
             <x14:dxf>
               <font>
@@ -2712,7 +2672,7 @@
           <xm:sqref>D12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{002E00F9-00FD-41D7-ADEB-00E400D30099}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{00B60089-007C-4D6F-8282-00DC007C00B4}">
             <xm:f>"Highest"</xm:f>
             <x14:dxf>
               <font>
@@ -2732,25 +2692,25 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4" disablePrompts="0">
-        <x14:dataValidation xr:uid="{0092002C-00C1-4979-82CC-002D004100C7}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{001F00AF-00D7-4ACB-A965-009E0045005F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Blocker,Critical,Major,Minor,Trivial"</xm:f>
           </x14:formula1>
           <xm:sqref>C2 C6</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{009100A3-00D6-4D6D-AF19-00B40043001B}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00AF008A-0027-428B-A27A-005100DA0013}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Highest,High,Medium,Low"</xm:f>
           </x14:formula1>
           <xm:sqref>D2 D6</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{003D002C-0075-4873-A4BD-005500B70075}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{008F008A-00C6-4BBD-8F8E-0085008A0089}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Blocker,Critical,Major,Minor,Trivial"</xm:f>
           </x14:formula1>
           <xm:sqref>C12</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{0061005A-00EF-4AF2-B913-007000540017}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00FF00C7-0083-44F1-9548-002E00DA00C1}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Highest,High,Medium,Low"</xm:f>
           </x14:formula1>

</xml_diff>